<commit_message>
Disable hydro using max capacity factor to reflect seasonal hydro variation.
</commit_message>
<xml_diff>
--- a/InputData/elec/BDTPTUMCF/Boolean Does This Plant Type Use Maximum Capacity Factor.xlsx
+++ b/InputData/elec/BDTPTUMCF/Boolean Does This Plant Type Use Maximum Capacity Factor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rod\Desktop\EPS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\Mexico\Models\eps-mexico\InputData\elec\BDTPTUMCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C31E864-8DCE-449D-AB96-BC2C9031E50D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C774EF9-87EB-49B3-AA0E-D9584FE0D8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="12" r:id="rId1"/>
@@ -162,7 +162,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -342,7 +342,7 @@
     <cellStyle name="Font: Calibri, 9pt regular" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Footnotes: top row" xfId="8" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Header: bottom row" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Hipervínculo" xfId="6" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="Normal 6" xfId="1" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
@@ -690,7 +690,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" customWidth="1"/>
     <col min="2" max="2" width="50.7109375" bestFit="1" customWidth="1"/>
@@ -698,15 +698,15 @@
     <col min="8" max="8" width="53.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -716,34 +716,34 @@
       <c r="E3" s="1"/>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="H7" s="4"/>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -765,20 +765,20 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.5703125" customWidth="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30">
+    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="7"/>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -787,7 +787,7 @@
       </c>
       <c r="C2" s="3"/>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -796,7 +796,7 @@
       </c>
       <c r="C3" s="3"/>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -805,7 +805,7 @@
       </c>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -814,16 +814,16 @@
       </c>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -832,7 +832,7 @@
       </c>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -841,7 +841,7 @@
       </c>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -850,7 +850,7 @@
       </c>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -859,7 +859,7 @@
       </c>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -868,7 +868,7 @@
       </c>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -877,7 +877,7 @@
       </c>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -886,7 +886,7 @@
       </c>
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -895,7 +895,7 @@
       </c>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -904,7 +904,7 @@
       </c>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -913,7 +913,7 @@
       </c>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -922,7 +922,7 @@
       </c>
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -931,7 +931,7 @@
       </c>
       <c r="C18" s="3"/>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -940,7 +940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -949,7 +949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -958,7 +958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -967,7 +967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>31</v>
       </c>
@@ -984,7 +984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>32</v>
       </c>
@@ -998,18 +998,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1157,13 +1157,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D950E80F-F787-4B60-9A57-C4CD2D907EFF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53E34236-7826-46C9-9B90-178B22EC10C2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53E34236-7826-46C9-9B90-178B22EC10C2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D950E80F-F787-4B60-9A57-C4CD2D907EFF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA834ED4-3D77-49C2-8CF2-DA77D70170D8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA834ED4-3D77-49C2-8CF2-DA77D70170D8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>